<commit_message>
feat: P4 Delivery/Impact Face 체인 추가 + Evidence Matrix 별점 반영
Top Geometry ↔ Evidence Matrix(Ball Flight) 연결 강화 (사용자 요청).

- 10개 Feature에 Delivery/Impact 예측 체인 추가:
  · Hand Height High/Low, Hand Depth Deep/Shallow,
    Lead Arm Plane Steep/Flat → [Medium] Shaft Plane→Club Delivery
  · Shaft Cross-Line → [Medium] Steep Shaft Delivery→Out-To-In
  · Shaft Laid Off → [Pattern Dependent] Shallow/Steep 분기
    (아마추어 Steep 케이스 반영)
  · Clubface Open/Closed Excessive → [Pattern Dependent]
    Impact Face 체인(At Impact / Late·Open 전략→Square)
- Ball Flight(Slice/Hook/Push/Pull 등)는 Feature Chain 미포함,
  Evidence Matrix에서만 관리 원칙 유지
- 사용자가 입력한 Evidence Matrix 별점(10 Feature × 6열) 반영

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L349258aAgr5FDzo3hWc1m
</commit_message>
<xml_diff>
--- a/DOH_P4.xlsx
+++ b/DOH_P4.xlsx
@@ -111,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -141,6 +141,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -641,7 +644,14 @@
 Branch C
 COM Elevation Continues
 ↓
-Early Extension (P6~P7)</t>
+Early Extension (P6~P7)
+[Medium Confidence] — Delivery / Evidence 연결
+Hand Height High (P4)
+↓
+Shaft Plane Steep (P5)
+↓
+Steep Club Delivery (P5~P6)
+(가파른 탑 구조가 가파른 클럽 전달로 이어진다.)</t>
         </is>
       </c>
     </row>
@@ -693,6 +703,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -793,7 +804,14 @@
 Branch C
 Inside Delivery Maintained
 ↓
-Inside Club Path (P6~P7)</t>
+Inside Club Path (P6~P7)
+[Medium Confidence] — Delivery / Evidence 연결
+Hand Height Low (P4)
+↓
+Shaft Plane Shallow (P5)
+↓
+Inside Club Delivery (P5~P6)
+(낮고 깊은 탑 구조가 인사이드 전달로 이어진다.)</t>
         </is>
       </c>
     </row>
@@ -845,6 +863,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
@@ -945,7 +964,14 @@
 Branch C
 Lead Knee Yields
 ↓
-Lead Knee Medial Collapse (P5~P6)</t>
+Lead Knee Medial Collapse (P5~P6)
+[Medium Confidence] — Delivery / Evidence 연결
+Hand Depth Deep (P4)
+↓
+Inside Club Delivery (P5~P6)
+↓
+Positive Attack Angle Tendency (P7)
+(깊은 손 구조가 인사이드 전달·어퍼블로 성향을 만든다. ※Positive AoA는 선택사항.)</t>
         </is>
       </c>
     </row>
@@ -997,6 +1023,7 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
@@ -1095,7 +1122,14 @@
 Branch C
 Steep Maintained
 ↓
-Low Point Variability (P7)</t>
+Low Point Variability (P7)
+[Medium Confidence] — Delivery / Evidence 연결
+Hand Depth Shallow (P4)
+↓
+Shaft Plane Steep (P5)
+↓
+Steep Club Delivery (P5~P6)
+(얕은 탑 구조가 가파른 클럽 전달로 이어진다.)</t>
         </is>
       </c>
     </row>
@@ -1145,6 +1179,7 @@
         </is>
       </c>
     </row>
+    <row r="34"/>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
@@ -1253,7 +1288,14 @@
 ↓
 Early Pelvis Open (P5~P6)
 ↓
-Spin-Out (P6)</t>
+Spin-Out (P6)
+[Medium Confidence] — Delivery / Evidence 연결
+Shaft Cross-Line (P4)
+↓
+Steep Shaft Delivery (P5)
+↓
+Out-To-In Club Delivery (P6)
+(아마추어에서 자주 나타나는 Steep·Out-To-In 전달 경로.)</t>
         </is>
       </c>
     </row>
@@ -1305,6 +1347,7 @@
         </is>
       </c>
     </row>
+    <row r="43"/>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
@@ -1402,7 +1445,21 @@
 Late Arm (P5)
 ↓
 Early Pelvis Open (P5~P6)
-※ Laid Off는 결과 체인 가중치를 낮게 둔다(우수 선수도 사용).</t>
+※ Laid Off는 결과 체인 가중치를 낮게 둔다(우수 선수도 사용).
+[Pattern Dependent] — Delivery / Evidence 연결
+Shaft Laid Off (P4)
+↓
+The Player Chooses A Different Delivery Strategy.
+(골퍼는 서로 다른 전달 전략을 선택한다.)
+Branch A
+Shallow Club Delivery (P5~P6)
+↓
+Inside Club Delivery (P6)
+Branch B
+The Player Chooses A Steep Delivery Strategy.
+↓
+Steep Club Delivery (P5~P6)
+※ 아마추어는 오히려 Steep으로 오는 경우가 많아 Branch로 관리한다.</t>
         </is>
       </c>
     </row>
@@ -1453,6 +1510,7 @@
         </is>
       </c>
     </row>
+    <row r="51"/>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
@@ -1559,7 +1617,18 @@
 Branch C
 Lag-Based Recovery
 ↓
-Release Pattern Change (P6)</t>
+Release Pattern Change (P6)
+[Pattern Dependent] — Impact Face / Evidence 연결
+Clubface Open Excessive (P4)
+↓
+Open Club Face At Impact (P7)
+Branch (Late Face Closure)
+Clubface Open Excessive (P4)
+↓
+The Player Chooses A Late Face Closure Strategy.
+↓
+Club Face Square At Impact (P7)
+※ Ball Flight(Slice/Push 등)는 Feature Chain에 포함하지 않고 Evidence Matrix에서만 관리.</t>
         </is>
       </c>
     </row>
@@ -1611,6 +1680,7 @@
         </is>
       </c>
     </row>
+    <row r="59"/>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
@@ -1717,7 +1787,18 @@
 Branch C
 Defensive Swing
 ↓
-Swing Speed Decrease (P7)</t>
+Swing Speed Decrease (P7)
+[Pattern Dependent] — Impact Face / Evidence 연결
+Clubface Closed Excessive (P4)
+↓
+Closed Club Face At Impact (P7)
+Branch (Open Delivery)
+Clubface Closed Excessive (P4)
+↓
+The Player Chooses An Open Delivery Strategy.
+↓
+Club Face Square At Impact (P7)
+※ Ball Flight(Hook/Pull 등)는 Feature Chain에 포함하지 않고 Evidence Matrix에서만 관리.</t>
         </is>
       </c>
     </row>
@@ -1768,6 +1849,7 @@
         </is>
       </c>
     </row>
+    <row r="67"/>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
@@ -1874,7 +1956,13 @@
 Branch C
 Steep Maintained
 ↓
-Low Point Variability (P7)</t>
+Low Point Variability (P7)
+[Medium Confidence] — Delivery / Evidence 연결
+Lead Arm Plane Steep (P4)
+↓
+Shaft Plane Steep (P5)
+↓
+Steep Club Delivery (P5~P6)</t>
         </is>
       </c>
     </row>
@@ -1924,6 +2012,7 @@
         </is>
       </c>
     </row>
+    <row r="76"/>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
@@ -2024,7 +2113,13 @@
 ↓
 Early Pelvis Open (P5~P6)
 ↓
-Spin-Out (P6)</t>
+Spin-Out (P6)
+[Medium Confidence] — Delivery / Evidence 연결
+Lead Arm Plane Flat (P4)
+↓
+Shaft Plane Shallow (P5)
+↓
+Inside Club Delivery (P5~P6)</t>
         </is>
       </c>
     </row>
@@ -2078,6 +2173,7 @@
         </is>
       </c>
     </row>
+    <row r="84"/>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
@@ -2227,6 +2323,7 @@
         </is>
       </c>
     </row>
+    <row r="92"/>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
@@ -2375,6 +2472,7 @@
         </is>
       </c>
     </row>
+    <row r="100"/>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
@@ -2533,6 +2631,7 @@
         </is>
       </c>
     </row>
+    <row r="108"/>
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
         <is>
@@ -2683,6 +2782,7 @@
         </is>
       </c>
     </row>
+    <row r="116"/>
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
         <is>
@@ -2835,6 +2935,7 @@
         </is>
       </c>
     </row>
+    <row r="124"/>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
@@ -2995,6 +3096,7 @@
         </is>
       </c>
     </row>
+    <row r="133"/>
     <row r="134">
       <c r="A134" s="4" t="inlineStr">
         <is>
@@ -3139,6 +3241,7 @@
         </is>
       </c>
     </row>
+    <row r="141"/>
     <row r="142">
       <c r="A142" s="4" t="inlineStr">
         <is>
@@ -3291,6 +3394,7 @@
         </is>
       </c>
     </row>
+    <row r="149"/>
     <row r="150">
       <c r="A150" s="4" t="inlineStr">
         <is>
@@ -3441,6 +3545,7 @@
         </is>
       </c>
     </row>
+    <row r="157"/>
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
         <is>
@@ -3583,6 +3688,7 @@
         </is>
       </c>
     </row>
+    <row r="165"/>
     <row r="166">
       <c r="A166" s="4" t="inlineStr">
         <is>
@@ -3727,6 +3833,7 @@
         </is>
       </c>
     </row>
+    <row r="173"/>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
@@ -3888,6 +3995,7 @@
         </is>
       </c>
     </row>
+    <row r="182"/>
     <row r="183">
       <c r="A183" s="4" t="inlineStr">
         <is>
@@ -4044,6 +4152,7 @@
         </is>
       </c>
     </row>
+    <row r="190"/>
     <row r="191">
       <c r="A191" s="4" t="inlineStr">
         <is>
@@ -4198,6 +4307,7 @@
         </is>
       </c>
     </row>
+    <row r="198"/>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
@@ -4360,6 +4470,7 @@
         </is>
       </c>
     </row>
+    <row r="207"/>
     <row r="208">
       <c r="A208" s="4" t="inlineStr">
         <is>
@@ -4512,6 +4623,7 @@
         </is>
       </c>
     </row>
+    <row r="215"/>
     <row r="216">
       <c r="A216" s="4" t="inlineStr">
         <is>
@@ -4664,6 +4776,7 @@
         </is>
       </c>
     </row>
+    <row r="223"/>
     <row r="224">
       <c r="A224" s="4" t="inlineStr">
         <is>
@@ -6443,7 +6556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -6745,6 +6858,23 @@
       <c r="C18" s="7" t="inlineStr">
         <is>
           <t>Thorax Rotation Insufficient·Head Height High 등 Hub Feature의 병렬 파생을 Chain이 아니라 DAG로 표현하는 스키마 확장. P5~P8 반복 확인 후. (Candidate 유지)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>DOH Chain Added</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Delivery / Impact Face 체인 (10 Feature)</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Hand Height High/Low · Hand Depth Deep/Shallow · Shaft Cross-Line · Lead Arm Plane Steep/Flat에 [Medium Confidence] Delivery 체인(→Shaft Plane→Club Delivery) 추가. Shaft Laid Off는 [Pattern Dependent](Shallow/Steep 분기, 아마추어 Steep 케이스). Clubface Open/Closed Excessive는 [Pattern Dependent] Impact Face 체인(→At Impact / Late·Open 전략→Square). Ball Flight는 Evidence Matrix에서만 관리. Top Geometry↔Evidence Matrix 연결 강화(사용자 요청).</t>
         </is>
       </c>
     </row>
@@ -11462,6 +11592,24 @@
           <t>Hand Height High (P4)</t>
         </is>
       </c>
+      <c r="F2" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="G2" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H2" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="I2" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="J2" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="K2" s="11" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -11469,6 +11617,24 @@
           <t>Hand Height Low (P4)</t>
         </is>
       </c>
+      <c r="F3" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="G3" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="H3" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="I3" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="J3" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="K3" s="11" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
@@ -11476,6 +11642,24 @@
           <t>Hand Depth Deep (P4)</t>
         </is>
       </c>
+      <c r="F4" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="G4" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="H4" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="I4" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="J4" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="K4" s="11" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -11483,6 +11667,24 @@
           <t>Hand Depth Shallow (P4)</t>
         </is>
       </c>
+      <c r="F5" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="G5" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="I5" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="J5" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="K5" s="11" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -11490,6 +11692,24 @@
           <t>Shaft Cross-Line (P4)</t>
         </is>
       </c>
+      <c r="F6" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H6" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="I6" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="J6" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="K6" s="11" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -11497,6 +11717,24 @@
           <t>Shaft Laid Off (P4)</t>
         </is>
       </c>
+      <c r="F7" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="G7" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="H7" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="I7" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="J7" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="K7" s="11" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -11504,6 +11742,24 @@
           <t>Clubface Open Excessive (P4)</t>
         </is>
       </c>
+      <c r="F8" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="G8" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="I8" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="J8" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="K8" s="11" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -11511,6 +11767,24 @@
           <t>Clubface Closed Excessive (P4)</t>
         </is>
       </c>
+      <c r="F9" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="H9" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="I9" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="J9" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="K9" s="11" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -11518,6 +11792,24 @@
           <t>Lead Arm Plane Steep (P4)</t>
         </is>
       </c>
+      <c r="F10" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="G10" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H10" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="I10" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="J10" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="K10" s="11" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -11525,6 +11817,24 @@
           <t>Lead Arm Plane Flat (P4)</t>
         </is>
       </c>
+      <c r="F11" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="G11" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="H11" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="I11" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="J11" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="K11" s="11" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -11652,6 +11962,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
         <is>
@@ -11662,7 +11973,7 @@
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>별점(★~-)은 이번 작업 범위 제외. P1~P8 설계 완료 후 별도 세션에서 일괄 부여.</t>
+          <t>Ball Flight 6열(Slice/Hook/Push/Pull/Fade/Draw)은 사용자가 Delivery 연계 10개 Feature에 대해 1차 입력(3~4). 나머지 접촉계열(Heel/Toe/High·Low Face/Fat/Thin/Top/Shank)과 잔여 Feature 별점은 P1~P8 설계 완료 후 별도 세션에서 일괄 부여.</t>
         </is>
       </c>
     </row>

</xml_diff>